<commit_message>
Zaman kuralı toplama anına bağlandı; fikstür yükleme zamanı (#93–#97)
- #93: İddaa kaydı Cuma (Salı) 17:00–19:00 TR; aralık dışı kayıt teste girmez
- #94: import-fixtures --uploaded-at zorunlu; önceki haftanın dosyası reddedilir
- #95: ±2 saat uyarısı kaldırıldı; referans dosya kaydın toplama gününe ait olmalı
- #96: dosyada referans oranı olmayan maç (Cuma akşamı) has_reference = 0, teste girmez
- #97: yükleme saati fixtures-log ile izlenir
- Şablon talimatları ve README güncellendi; tzdata bağımlılığı (Windows)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/iddaa_kayit_sablonu.xlsx
+++ b/templates/iddaa_kayit_sablonu.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="110" customWidth="1" style="14" min="1" max="1"/>
@@ -582,99 +582,113 @@
     <row r="1" ht="15" customHeight="1" s="15">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>İddaa kayıt şablonu – tek kaynak (karar #79). Faz 8.1, 8.2, 8.7 ve Faz 12 kayıtları buradan girilir.</t>
+          <t>İddaa kayıt şablonu – tek kaynak (karar #79). Zaman kuralları: #93–#96.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="15">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Ne zaman: Her Cuma 18:00–20:00 arası (TR saati). Hafta içi maçlar için Salı aynı saatler.</t>
+          <t>CUMA 17:00–19:00 (TR saati; hafta içi maçlar için SALI aynı saatler): İddaa oranlarını gir.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>1. football-data'dan fixtures.csv dosyasını indir. Üzerine yazma; tarih ve saatle adlandır: fixtures_YYYYAAGG_SSDD.csv</t>
+          <t xml:space="preserve">  Bu aralık football-data'nın oranları topladığı öğleden sonraya denk gelir (İngiltere saatiyle 15–17, 25 Ekim'den sonra 14–16).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="15">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>2. Dosyayı yükle:  betsistem import-fixtures fixtures_YYYYAAGG_SSDD.csv   (sha ve indirme zamanı kaydedilir)</t>
+          <t xml:space="preserve">  Hafta sonu oynanacak her E0 ve T1 maçı için 1, X, 2 oranları ve MBS. kayit_zamani: oranları gördüğün an. Aralık dışı kayıt teste girmez.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="15">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>3. İddaa bültenini aç. Hafta sonu oynanacak her E0 ve T1 maçı için 1, X, 2 oranlarını ve MBS sayısını gir.</t>
+          <t>CUMARTESİ SABAH (yükleme sonrası): football-data'dan fixtures.csv dosyasını indir.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="15">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>4. kayit_zamani: oranları gördüğün an (TR saati). Fikstür dosyasının indirilmesinden en çok 2 saat önce/sonra (karar #76).</t>
+          <t xml:space="preserve">  Sitedeki 'Latest fixtures uploaded' zamanını not et (ör. 24/10/26 09:35). Dosyayı fixtures_YYYYAAGG_SSDD.csv diye kaydet.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="15">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>5. Takım adları football-data yazımıyla: fikstür dosyasındaki HomeTeam/AwayTeam ile birebir aynı (ör. Man United, Nott'm Forest).</t>
+          <t xml:space="preserve">  Yükle:  betsistem import-fixtures fixtures_20261024_1000.csv --uploaded-at "24/10/26 09:35"</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Yardım için 'Takımlar' sayfasına bak. İçe aktarma her satırı fikstür dosyasındaki maçla eşleştirir; yazım yanlışsa öneri verir.</t>
+          <t xml:space="preserve">  Site hâlâ önceki haftanın yüklemesini gösteriyorsa dosya reddedilir; yeni yüklemeyi bekle (#94).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="15">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>6. fikstur_dosyasi sütununa 1. adımdaki dosya adını aynen yaz.</t>
+          <t>fikstur_dosyasi sütununa bu dosyanın adını yaz (Cuma kayıtları, ertesi sabah yüklenen o haftanın dosyasına bağlanır).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>7. Ondalık için virgül ya da nokta kullanabilirsin (1,85 veya 1.85).</t>
+          <t>Takım adları football-data yazımıyla (ör. Man United, Nott'm Forest); 'Takımlar' sayfasına bak. Yanlış yazımda öneri verilir.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>8. Oran değişse bile eski satırı düzeltme; yeni kayıt yeni satırdır. Dosyayı birikimli tutabilirsin.</t>
+          <t>Cuma akşamı oynanan maçları da gir: dosyada yer almadıkları için teste girmezler ama MBS ve marj ölçümünde kullanılırlar (#96).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>9. Kaydet ve yükle:  betsistem import-iddaa &lt;dosya&gt;.xlsx   (önceki satırlar atlanır; hatalı satır varsa hiçbir şey yazılmaz)</t>
+          <t>Ondalık için virgül ya da nokta kullanabilirsin (1,85 veya 1.85). MBS tam sayı.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Oran değişse bile eski satırı düzeltme; yeni kayıt yeni satırdır. Dosyayı birikimli tutabilirsin.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Örnek satır: 2026-10-23 19:40 | E0 | 2026-10-24 | 17:00 | Arsenal | Chelsea | 1,85 | 3,60 | 4,10 | 1 | fixtures_20261023_1930.csv |</t>
+          <t>Yükle:  betsistem import-iddaa &lt;dosya&gt;.xlsx   (önceki satırlar atlanır; hatalı satır varsa hiçbir şey yazılmaz)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Örnek satır: 2026-10-23 17:40 | E0 | 2026-10-24 | 17:00 | Arsenal | Chelsea | 1,85 | 3,60 | 4,10 | 1 | fixtures_20261024_1000.csv |</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Özet sayfası her lig için MBS 1 oranını ve ortalama İddaa marjını hesaplar. Sarı hücreleri sen doldurursun; iddaa_marji otomatik.</t>
         </is>
@@ -9940,235 +9954,235 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Arsenal</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Ad. Demirspor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Alanyaspor</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Bournemouth</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Ankaragucu</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Brentford</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Antalyaspor</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Brighton</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Besiktas</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Chelsea</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Buyuksehyr</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Coventry</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Fenerbahce</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Crystal Palace</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Galatasaray</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Everton</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Gaziantep</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Fulham</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Giresunspor</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Hull</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Hatayspor</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Ipswich</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Istanbulspor</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Karagumruk</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Liverpool</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Kasimpasa</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Man City</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Kayserispor</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Man United</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>Konyaspor</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Newcastle</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Sivasspor</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Nott'm Forest</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Trabzonspor</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Sunderland</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Umraniyespor</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Tottenham</t>
         </is>

</xml_diff>